<commit_message>
Update category_map.xlsx via NBS Ad Tracker
</commit_message>
<xml_diff>
--- a/category_map.xlsx
+++ b/category_map.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -17,16 +17,13 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="2">
+  <fonts count="1">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
-    </font>
-    <font>
-      <b val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -37,7 +34,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -45,21 +42,12 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin"/>
-      <right style="thin"/>
-      <top style="thin"/>
-      <bottom style="thin"/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -425,46 +413,46 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H427"/>
+  <dimension ref="A1:H432"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>AD Name</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>Category</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>AD/SQ Type</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>Times Seen</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>Category Consistent</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>Last Updated</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>Updated By</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t>Notes</t>
         </is>
@@ -15927,6 +15915,206 @@
       <c r="H427" t="inlineStr">
         <is>
           <t>Added via Mapping Manager</t>
+        </is>
+      </c>
+    </row>
+    <row r="428">
+      <c r="A428" t="inlineStr">
+        <is>
+          <t>AFRO CINEMA</t>
+        </is>
+      </c>
+      <c r="B428" t="inlineStr">
+        <is>
+          <t>Internal</t>
+        </is>
+      </c>
+      <c r="C428" t="inlineStr">
+        <is>
+          <t>AD</t>
+        </is>
+      </c>
+      <c r="D428" t="n">
+        <v>1</v>
+      </c>
+      <c r="E428" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="F428" t="inlineStr">
+        <is>
+          <t>20.07.2026</t>
+        </is>
+      </c>
+      <c r="G428" t="inlineStr">
+        <is>
+          <t>App User</t>
+        </is>
+      </c>
+      <c r="H428" t="inlineStr">
+        <is>
+          <t>Added via Assign Categories</t>
+        </is>
+      </c>
+    </row>
+    <row r="429">
+      <c r="A429" t="inlineStr">
+        <is>
+          <t>CREATA HUB</t>
+        </is>
+      </c>
+      <c r="B429" t="inlineStr">
+        <is>
+          <t>Internal</t>
+        </is>
+      </c>
+      <c r="C429" t="inlineStr">
+        <is>
+          <t>AD</t>
+        </is>
+      </c>
+      <c r="D429" t="n">
+        <v>1</v>
+      </c>
+      <c r="E429" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="F429" t="inlineStr">
+        <is>
+          <t>20.07.2026</t>
+        </is>
+      </c>
+      <c r="G429" t="inlineStr">
+        <is>
+          <t>App User</t>
+        </is>
+      </c>
+      <c r="H429" t="inlineStr">
+        <is>
+          <t>Added via Assign Categories</t>
+        </is>
+      </c>
+    </row>
+    <row r="430">
+      <c r="A430" t="inlineStr">
+        <is>
+          <t>HONOURABLES</t>
+        </is>
+      </c>
+      <c r="B430" t="inlineStr">
+        <is>
+          <t>Internal</t>
+        </is>
+      </c>
+      <c r="C430" t="inlineStr">
+        <is>
+          <t>AD</t>
+        </is>
+      </c>
+      <c r="D430" t="n">
+        <v>1</v>
+      </c>
+      <c r="E430" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="F430" t="inlineStr">
+        <is>
+          <t>20.07.2026</t>
+        </is>
+      </c>
+      <c r="G430" t="inlineStr">
+        <is>
+          <t>App User</t>
+        </is>
+      </c>
+      <c r="H430" t="inlineStr">
+        <is>
+          <t>Added via Assign Categories</t>
+        </is>
+      </c>
+    </row>
+    <row r="431">
+      <c r="A431" t="inlineStr">
+        <is>
+          <t>LIVE NBS AT EIGHNTEEN</t>
+        </is>
+      </c>
+      <c r="B431" t="inlineStr">
+        <is>
+          <t>Internal</t>
+        </is>
+      </c>
+      <c r="C431" t="inlineStr">
+        <is>
+          <t>AD</t>
+        </is>
+      </c>
+      <c r="D431" t="n">
+        <v>1</v>
+      </c>
+      <c r="E431" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="F431" t="inlineStr">
+        <is>
+          <t>20.07.2026</t>
+        </is>
+      </c>
+      <c r="G431" t="inlineStr">
+        <is>
+          <t>App User</t>
+        </is>
+      </c>
+      <c r="H431" t="inlineStr">
+        <is>
+          <t>Added via Assign Categories</t>
+        </is>
+      </c>
+    </row>
+    <row r="432">
+      <c r="A432" t="inlineStr">
+        <is>
+          <t>PROMO NILE RESORT</t>
+        </is>
+      </c>
+      <c r="B432" t="inlineStr">
+        <is>
+          <t>Internal</t>
+        </is>
+      </c>
+      <c r="C432" t="inlineStr">
+        <is>
+          <t>AD</t>
+        </is>
+      </c>
+      <c r="D432" t="n">
+        <v>1</v>
+      </c>
+      <c r="E432" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="F432" t="inlineStr">
+        <is>
+          <t>20.07.2026</t>
+        </is>
+      </c>
+      <c r="G432" t="inlineStr">
+        <is>
+          <t>App User</t>
+        </is>
+      </c>
+      <c r="H432" t="inlineStr">
+        <is>
+          <t>Added via Assign Categories</t>
         </is>
       </c>
     </row>

</xml_diff>